<commit_message>
Phase AO: the input workbooks the website offers carry Break Set For Shifts Of 11 Hours Or More = 15, 30, 15, 15 (four breaks for an 11-hour shift)
The engine already reads this row (audit F-20); shorter shifts keep their own set. The staged test that
compares the Example with its source is re-pinned with the row added to the source, and says why.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012jkpuBfug5TnsMSqQWAuNe
</commit_message>
<xml_diff>
--- a/webapp/workbooks/Scheduler_Input_Blank.xlsx
+++ b/webapp/workbooks/Scheduler_Input_Blank.xlsx
@@ -6729,7 +6729,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="18" min="1" max="1"/>
@@ -7451,132 +7451,149 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="40" t="inlineStr">
+    <row r="57" ht="20" customHeight="1" s="18">
+      <c r="B57" s="42" t="inlineStr">
+        <is>
+          <t>Break Set For Shifts Of 11 Hours Or More</t>
+        </is>
+      </c>
+      <c r="C57" s="43" t="inlineStr">
+        <is>
+          <t>15, 30, 15, 15</t>
+        </is>
+      </c>
+      <c r="D57" s="44" t="inlineStr">
+        <is>
+          <t>Shifts of 11 hours or more get these breaks in this order, in minutes (30 or more is a lunch): 15, 30, 15, 15 = two short breaks around a lunch, then one more. Shorter shifts keep the counts above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="40" t="inlineStr">
         <is>
           <t>Language / Skill</t>
         </is>
       </c>
-      <c r="B58" s="41" t="n"/>
-      <c r="C58" s="41" t="n"/>
-      <c r="D58" s="41" t="n"/>
-    </row>
-    <row r="59" ht="20" customHeight="1" s="18">
-      <c r="B59" s="42" t="inlineStr">
+      <c r="B59" s="41" t="n"/>
+      <c r="C59" s="41" t="n"/>
+      <c r="D59" s="41" t="n"/>
+    </row>
+    <row r="60" ht="20" customHeight="1" s="18">
+      <c r="B60" s="42" t="inlineStr">
         <is>
           <t>Language Working Window</t>
         </is>
       </c>
-      <c r="C59" s="43" t="inlineStr"/>
-      <c r="D59" s="44" t="inlineStr">
+      <c r="C60" s="43" t="inlineStr"/>
+      <c r="D60" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. OFF = language hours set minimums only. The other choices also limit when each language may work (guide 3.7).</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="40" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="40" t="inlineStr">
         <is>
           <t>Exception Policy</t>
         </is>
       </c>
-      <c r="B61" s="41" t="n"/>
-      <c r="C61" s="41" t="n"/>
-      <c r="D61" s="41" t="n"/>
-    </row>
-    <row r="62" ht="20" customHeight="1" s="18">
-      <c r="B62" s="42" t="inlineStr">
-        <is>
-          <t>Critical Coverage No-Break Exception Enabled</t>
-        </is>
-      </c>
-      <c r="C62" s="43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D62" s="44" t="inlineStr">
-        <is>
-          <t>Yes = a person may skip a break when coverage is critical (set a limit below).</t>
-        </is>
-      </c>
+      <c r="B62" s="41" t="n"/>
+      <c r="C62" s="41" t="n"/>
+      <c r="D62" s="41" t="n"/>
     </row>
     <row r="63" ht="20" customHeight="1" s="18">
       <c r="B63" s="42" t="inlineStr">
         <is>
+          <t>Critical Coverage No-Break Exception Enabled</t>
+        </is>
+      </c>
+      <c r="C63" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D63" s="44" t="inlineStr">
+        <is>
+          <t>Yes = a person may skip a break when coverage is critical (set a limit below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1" s="18">
+      <c r="B64" s="42" t="inlineStr">
+        <is>
           <t>Critical Coverage No-Break Max Associate-Days</t>
         </is>
       </c>
-      <c r="C63" s="45" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="44" t="inlineStr">
+      <c r="C64" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="44" t="inlineStr">
         <is>
           <t>Most person-days that may skip a break. Above 0 when enabled.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="40" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="40" t="inlineStr">
         <is>
           <t>Release Quality   (click + on the left to open)</t>
         </is>
       </c>
-      <c r="B65" s="41" t="n"/>
-      <c r="C65" s="41" t="n"/>
-      <c r="D65" s="41" t="n"/>
-    </row>
-    <row r="66" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B66" s="42" t="inlineStr">
-        <is>
-          <t>Production Quality Gate Mode</t>
-        </is>
-      </c>
-      <c r="C66" s="43" t="inlineStr">
-        <is>
-          <t>Warn</t>
-        </is>
-      </c>
-      <c r="D66" s="44" t="inlineStr">
-        <is>
-          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
-        </is>
-      </c>
+      <c r="B66" s="41" t="n"/>
+      <c r="C66" s="41" t="n"/>
+      <c r="D66" s="41" t="n"/>
     </row>
     <row r="67" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B67" s="42" t="inlineStr">
         <is>
-          <t>Minimum After Break Target Ratio</t>
-        </is>
-      </c>
-      <c r="C67" s="46" t="inlineStr"/>
+          <t>Production Quality Gate Mode</t>
+        </is>
+      </c>
+      <c r="C67" s="43" t="inlineStr">
+        <is>
+          <t>Warn</t>
+        </is>
+      </c>
       <c r="D67" s="44" t="inlineStr">
         <is>
-          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
+          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
         </is>
       </c>
     </row>
     <row r="68" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B68" s="42" t="inlineStr">
         <is>
-          <t>Protected Before80 Minimum Intervals</t>
-        </is>
-      </c>
-      <c r="C68" s="45" t="inlineStr"/>
+          <t>Minimum After Break Target Ratio</t>
+        </is>
+      </c>
+      <c r="C68" s="46" t="inlineStr"/>
       <c r="D68" s="44" t="inlineStr">
         <is>
-          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
+          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
         </is>
       </c>
     </row>
     <row r="69" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B69" s="42" t="inlineStr">
         <is>
-          <t>Protected After80 Minimum Intervals</t>
+          <t>Protected Before80 Minimum Intervals</t>
         </is>
       </c>
       <c r="C69" s="45" t="inlineStr"/>
       <c r="D69" s="44" t="inlineStr">
+        <is>
+          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B70" s="42" t="inlineStr">
+        <is>
+          <t>Protected After80 Minimum Intervals</t>
+        </is>
+      </c>
+      <c r="C70" s="45" t="inlineStr"/>
+      <c r="D70" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. Optional. Intervals that must reach 80% after breaks.</t>
         </is>
@@ -7587,7 +7604,7 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <dataValidations count="31">
+  <dataValidations count="32">
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 80 characters." prompt="Up to 80 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
       <formula1>80</formula1>
     </dataValidation>
@@ -7595,7 +7612,7 @@
       <formula1>1</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C8 C16 C20 C22 C28 C30 C31 C34 C37 C38 C39 C40 C44 C56 C62" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C8 C16 C20 C22 C28 C30 C31 C34 C37 C38 C39 C40 C44 C56 C63" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
@@ -7674,25 +7691,28 @@
       <formula1>0</formula1>
       <formula2>720</formula2>
     </dataValidation>
-    <dataValidation sqref="C59" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C57" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 40 characters." prompt="Up to 40 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
+      <formula1>40</formula1>
+    </dataValidation>
+    <dataValidation sqref="C60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"OFF,MINIMUM_ROWS,ALL_ROWS,REQUIRED_LANGUAGE_ONLY"</formula1>
     </dataValidation>
-    <dataValidation sqref="C63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C66" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C67" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Warn,Fail,Off"</formula1>
     </dataValidation>
-    <dataValidation sqref="C67" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="C68" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="C68" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C69" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>
-    <dataValidation sqref="C69" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C70" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Phase AQ: the shift-rule row in the website's input workbooks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012jkpuBfug5TnsMSqQWAuNe
</commit_message>
<xml_diff>
--- a/webapp/workbooks/Scheduler_Input_Blank.xlsx
+++ b/webapp/workbooks/Scheduler_Input_Blank.xlsx
@@ -6729,7 +6729,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="18" min="1" max="1"/>
@@ -7491,109 +7491,126 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="40" t="inlineStr">
+    <row r="61" ht="20" customHeight="1" s="18">
+      <c r="B61" s="42" t="inlineStr">
+        <is>
+          <t>Language Working Window Shift Rule</t>
+        </is>
+      </c>
+      <c r="C61" s="43" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="D61" s="44" t="inlineStr">
+        <is>
+          <t>START = a shift only has to begin inside the language window (the default). WHOLE_SHIFT = it must begin and end inside it. Used only when Language Working Window above is not OFF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="40" t="inlineStr">
         <is>
           <t>Exception Policy</t>
         </is>
       </c>
-      <c r="B62" s="41" t="n"/>
-      <c r="C62" s="41" t="n"/>
-      <c r="D62" s="41" t="n"/>
-    </row>
-    <row r="63" ht="20" customHeight="1" s="18">
-      <c r="B63" s="42" t="inlineStr">
-        <is>
-          <t>Critical Coverage No-Break Exception Enabled</t>
-        </is>
-      </c>
-      <c r="C63" s="43" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D63" s="44" t="inlineStr">
-        <is>
-          <t>Yes = a person may skip a break when coverage is critical (set a limit below).</t>
-        </is>
-      </c>
+      <c r="B63" s="41" t="n"/>
+      <c r="C63" s="41" t="n"/>
+      <c r="D63" s="41" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1" s="18">
       <c r="B64" s="42" t="inlineStr">
         <is>
+          <t>Critical Coverage No-Break Exception Enabled</t>
+        </is>
+      </c>
+      <c r="C64" s="43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D64" s="44" t="inlineStr">
+        <is>
+          <t>Yes = a person may skip a break when coverage is critical (set a limit below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1" s="18">
+      <c r="B65" s="42" t="inlineStr">
+        <is>
           <t>Critical Coverage No-Break Max Associate-Days</t>
         </is>
       </c>
-      <c r="C64" s="45" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" s="44" t="inlineStr">
+      <c r="C65" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="44" t="inlineStr">
         <is>
           <t>Most person-days that may skip a break. Above 0 when enabled.</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="40" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="40" t="inlineStr">
         <is>
           <t>Release Quality   (click + on the left to open)</t>
         </is>
       </c>
-      <c r="B66" s="41" t="n"/>
-      <c r="C66" s="41" t="n"/>
-      <c r="D66" s="41" t="n"/>
-    </row>
-    <row r="67" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B67" s="42" t="inlineStr">
-        <is>
-          <t>Production Quality Gate Mode</t>
-        </is>
-      </c>
-      <c r="C67" s="43" t="inlineStr">
-        <is>
-          <t>Warn</t>
-        </is>
-      </c>
-      <c r="D67" s="44" t="inlineStr">
-        <is>
-          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
-        </is>
-      </c>
+      <c r="B67" s="41" t="n"/>
+      <c r="C67" s="41" t="n"/>
+      <c r="D67" s="41" t="n"/>
     </row>
     <row r="68" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B68" s="42" t="inlineStr">
         <is>
-          <t>Minimum After Break Target Ratio</t>
-        </is>
-      </c>
-      <c r="C68" s="46" t="inlineStr"/>
+          <t>Production Quality Gate Mode</t>
+        </is>
+      </c>
+      <c r="C68" s="43" t="inlineStr">
+        <is>
+          <t>Warn</t>
+        </is>
+      </c>
       <c r="D68" s="44" t="inlineStr">
         <is>
-          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
+          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
         </is>
       </c>
     </row>
     <row r="69" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B69" s="42" t="inlineStr">
         <is>
-          <t>Protected Before80 Minimum Intervals</t>
-        </is>
-      </c>
-      <c r="C69" s="45" t="inlineStr"/>
+          <t>Minimum After Break Target Ratio</t>
+        </is>
+      </c>
+      <c r="C69" s="46" t="inlineStr"/>
       <c r="D69" s="44" t="inlineStr">
         <is>
-          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
+          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
         </is>
       </c>
     </row>
     <row r="70" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B70" s="42" t="inlineStr">
         <is>
-          <t>Protected After80 Minimum Intervals</t>
+          <t>Protected Before80 Minimum Intervals</t>
         </is>
       </c>
       <c r="C70" s="45" t="inlineStr"/>
       <c r="D70" s="44" t="inlineStr">
+        <is>
+          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B71" s="42" t="inlineStr">
+        <is>
+          <t>Protected After80 Minimum Intervals</t>
+        </is>
+      </c>
+      <c r="C71" s="45" t="inlineStr"/>
+      <c r="D71" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. Optional. Intervals that must reach 80% after breaks.</t>
         </is>
@@ -7604,7 +7621,7 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <dataValidations count="32">
+  <dataValidations count="33">
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 80 characters." prompt="Up to 80 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
       <formula1>80</formula1>
     </dataValidation>
@@ -7612,7 +7629,7 @@
       <formula1>1</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C8 C16 C20 C22 C28 C30 C31 C34 C37 C38 C39 C40 C44 C56 C63" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C8 C16 C20 C22 C28 C30 C31 C34 C37 C38 C39 C40 C44 C56 C64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
@@ -7697,22 +7714,25 @@
     <dataValidation sqref="C60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"OFF,MINIMUM_ROWS,ALL_ROWS,REQUIRED_LANGUAGE_ONLY"</formula1>
     </dataValidation>
-    <dataValidation sqref="C64" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C61" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+      <formula1>"START,WHOLE_SHIFT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C65" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C67" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C68" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Warn,Fail,Off"</formula1>
     </dataValidation>
-    <dataValidation sqref="C68" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="C69" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="C69" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C70" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>
-    <dataValidation sqref="C70" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C71" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Blank and example workbooks show the limit on breaks at once: count, share and gate mode in the Breaks group
They were on the hidden Engine Defaults sheet, so the limit (4 at a time, 30%, Warn) was invisible. The visible rows show the same defaults, so nothing changes until they are edited.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012jkpuBfug5TnsMSqQWAuNe
</commit_message>
<xml_diff>
--- a/webapp/workbooks/Scheduler_Input_Blank.xlsx
+++ b/webapp/workbooks/Scheduler_Input_Blank.xlsx
@@ -6729,7 +6729,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D71"/>
+  <dimension ref="A1:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="18" min="1" max="1"/>
@@ -7468,149 +7468,196 @@
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="40" t="inlineStr">
-        <is>
-          <t>Language / Skill</t>
-        </is>
-      </c>
-      <c r="B59" s="41" t="n"/>
-      <c r="C59" s="41" t="n"/>
-      <c r="D59" s="41" t="n"/>
+    <row r="58" ht="20" customHeight="1" s="18">
+      <c r="B58" s="42" t="inlineStr">
+        <is>
+          <t>Maximum Concurrent Break Ratio</t>
+        </is>
+      </c>
+      <c r="C58" s="46" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D58" s="44" t="inlineStr">
+        <is>
+          <t>Most share of the people on shift on a break at once, like 30% or 0.30. Blank = 30%. Kept between 5% and 75%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1" s="18">
+      <c r="B59" s="42" t="inlineStr">
+        <is>
+          <t>Maximum Concurrent Breaks</t>
+        </is>
+      </c>
+      <c r="C59" s="45" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" s="44" t="inlineStr">
+        <is>
+          <t>Most people on a break at the same time. Blank = 4. Not above one less than the people on shift.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="20" customHeight="1" s="18">
       <c r="B60" s="42" t="inlineStr">
         <is>
+          <t>Break Concurrency Gate Mode</t>
+        </is>
+      </c>
+      <c r="C60" s="43" t="inlineStr">
+        <is>
+          <t>Warn</t>
+        </is>
+      </c>
+      <c r="D60" s="44" t="inlineStr">
+        <is>
+          <t>Warn = more breaks at once than the limit costs about as much as a missed target interval (the default). Fail = never more than the limit. Off = no limit on breaks at once: intervals decide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="40" t="inlineStr">
+        <is>
+          <t>Language / Skill</t>
+        </is>
+      </c>
+      <c r="B62" s="41" t="n"/>
+      <c r="C62" s="41" t="n"/>
+      <c r="D62" s="41" t="n"/>
+    </row>
+    <row r="63" ht="20" customHeight="1" s="18">
+      <c r="B63" s="42" t="inlineStr">
+        <is>
           <t>Language Working Window</t>
         </is>
       </c>
-      <c r="C60" s="43" t="inlineStr"/>
-      <c r="D60" s="44" t="inlineStr">
+      <c r="C63" s="43" t="inlineStr"/>
+      <c r="D63" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. OFF = language hours set minimums only. The other choices also limit when each language may work (guide 3.7).</t>
         </is>
       </c>
-    </row>
-    <row r="61" ht="20" customHeight="1" s="18">
-      <c r="B61" s="42" t="inlineStr">
-        <is>
-          <t>Language Working Window Shift Rule</t>
-        </is>
-      </c>
-      <c r="C61" s="43" t="inlineStr">
-        <is>
-          <t>START</t>
-        </is>
-      </c>
-      <c r="D61" s="44" t="inlineStr">
-        <is>
-          <t>START = a shift only has to begin inside the language window (the default). WHOLE_SHIFT = it must begin and end inside it. Used only when Language Working Window above is not OFF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="40" t="inlineStr">
-        <is>
-          <t>Exception Policy</t>
-        </is>
-      </c>
-      <c r="B63" s="41" t="n"/>
-      <c r="C63" s="41" t="n"/>
-      <c r="D63" s="41" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1" s="18">
       <c r="B64" s="42" t="inlineStr">
         <is>
+          <t>Language Working Window Shift Rule</t>
+        </is>
+      </c>
+      <c r="C64" s="43" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="D64" s="44" t="inlineStr">
+        <is>
+          <t>START = a shift only has to begin inside the language window (the default). WHOLE_SHIFT = it must begin and end inside it. Used only when Language Working Window above is not OFF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="40" t="inlineStr">
+        <is>
+          <t>Exception Policy</t>
+        </is>
+      </c>
+      <c r="B66" s="41" t="n"/>
+      <c r="C66" s="41" t="n"/>
+      <c r="D66" s="41" t="n"/>
+    </row>
+    <row r="67" ht="20" customHeight="1" s="18">
+      <c r="B67" s="42" t="inlineStr">
+        <is>
           <t>Critical Coverage No-Break Exception Enabled</t>
         </is>
       </c>
-      <c r="C64" s="43" t="inlineStr">
+      <c r="C67" s="43" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D64" s="44" t="inlineStr">
+      <c r="D67" s="44" t="inlineStr">
         <is>
           <t>Yes = a person may skip a break when coverage is critical (set a limit below).</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="20" customHeight="1" s="18">
-      <c r="B65" s="42" t="inlineStr">
+    <row r="68" ht="20" customHeight="1" s="18">
+      <c r="B68" s="42" t="inlineStr">
         <is>
           <t>Critical Coverage No-Break Max Associate-Days</t>
         </is>
       </c>
-      <c r="C65" s="45" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" s="44" t="inlineStr">
+      <c r="C68" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="44" t="inlineStr">
         <is>
           <t>Most person-days that may skip a break. Above 0 when enabled.</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="40" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="40" t="inlineStr">
         <is>
           <t>Release Quality   (click + on the left to open)</t>
         </is>
       </c>
-      <c r="B67" s="41" t="n"/>
-      <c r="C67" s="41" t="n"/>
-      <c r="D67" s="41" t="n"/>
-    </row>
-    <row r="68" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B68" s="42" t="inlineStr">
-        <is>
-          <t>Production Quality Gate Mode</t>
-        </is>
-      </c>
-      <c r="C68" s="43" t="inlineStr">
-        <is>
-          <t>Warn</t>
-        </is>
-      </c>
-      <c r="D68" s="44" t="inlineStr">
-        <is>
-          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B69" s="42" t="inlineStr">
-        <is>
-          <t>Minimum After Break Target Ratio</t>
-        </is>
-      </c>
-      <c r="C69" s="46" t="inlineStr"/>
-      <c r="D69" s="44" t="inlineStr">
-        <is>
-          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
-      <c r="B70" s="42" t="inlineStr">
-        <is>
-          <t>Protected Before80 Minimum Intervals</t>
-        </is>
-      </c>
-      <c r="C70" s="45" t="inlineStr"/>
-      <c r="D70" s="44" t="inlineStr">
-        <is>
-          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
-        </is>
-      </c>
+      <c r="B70" s="41" t="n"/>
+      <c r="C70" s="41" t="n"/>
+      <c r="D70" s="41" t="n"/>
     </row>
     <row r="71" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
       <c r="B71" s="42" t="inlineStr">
         <is>
+          <t>Production Quality Gate Mode</t>
+        </is>
+      </c>
+      <c r="C71" s="43" t="inlineStr">
+        <is>
+          <t>Warn</t>
+        </is>
+      </c>
+      <c r="D71" s="44" t="inlineStr">
+        <is>
+          <t>Warn = report quality issues. Fail = block release. Off = ignore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B72" s="42" t="inlineStr">
+        <is>
+          <t>Minimum After Break Target Ratio</t>
+        </is>
+      </c>
+      <c r="C72" s="46" t="inlineStr"/>
+      <c r="D72" s="44" t="inlineStr">
+        <is>
+          <t>Blank = engine default. Optional. Lowest share of intervals at target after breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B73" s="42" t="inlineStr">
+        <is>
+          <t>Protected Before80 Minimum Intervals</t>
+        </is>
+      </c>
+      <c r="C73" s="45" t="inlineStr"/>
+      <c r="D73" s="44" t="inlineStr">
+        <is>
+          <t>Blank = engine default. Optional. Intervals that must reach 80% before breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" hidden="1" outlineLevel="1" ht="20" customHeight="1" s="18">
+      <c r="B74" s="42" t="inlineStr">
+        <is>
           <t>Protected After80 Minimum Intervals</t>
         </is>
       </c>
-      <c r="C71" s="45" t="inlineStr"/>
-      <c r="D71" s="44" t="inlineStr">
+      <c r="C74" s="45" t="inlineStr"/>
+      <c r="D74" s="44" t="inlineStr">
         <is>
           <t>Blank = engine default. Optional. Intervals that must reach 80% after breaks.</t>
         </is>
@@ -7621,7 +7668,7 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <dataValidations count="33">
+  <dataValidations count="35">
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 80 characters." prompt="Up to 80 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
       <formula1>80</formula1>
     </dataValidation>
@@ -7629,7 +7676,7 @@
       <formula1>1</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C8 C16 C20 C22 C28 C30 C31 C34 C37 C38 C39 C40 C44 C56 C64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C8 C16 C20 C22 C28 C30 C31 C34 C37 C38 C39 C40 C44 C56 C67" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
@@ -7711,28 +7758,36 @@
     <dataValidation sqref="C57" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Up to 40 characters." prompt="Up to 40 characters." type="textLength" errorStyle="stop" operator="lessThanOrEqual">
       <formula1>40</formula1>
     </dataValidation>
-    <dataValidation sqref="C60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C58" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation sqref="C59" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 1 to 5000." prompt="Enter a whole number from 1 to 5000." type="whole" errorStyle="stop" operator="between">
+      <formula1>1</formula1>
+      <formula2>5000</formula2>
+    </dataValidation>
+    <dataValidation sqref="C60 C71" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+      <formula1>"Warn,Fail,Off"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C63" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"OFF,MINIMUM_ROWS,ALL_ROWS,REQUIRED_LANGUAGE_ONLY"</formula1>
     </dataValidation>
-    <dataValidation sqref="C61" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"START,WHOLE_SHIFT"</formula1>
     </dataValidation>
-    <dataValidation sqref="C65" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C68" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 5000." prompt="Enter a whole number from 0 to 5000." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>5000</formula2>
     </dataValidation>
-    <dataValidation sqref="C68" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
-      <formula1>"Warn,Fail,Off"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C69" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="C72" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="C70" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C73" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>
-    <dataValidation sqref="C71" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C74" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>
@@ -13043,7 +13098,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="18" min="1" max="1"/>
@@ -13210,7 +13265,7 @@
     <row r="18">
       <c r="A18" s="40" t="inlineStr">
         <is>
-          <t>Break Concurrency</t>
+          <t>Week Boundary</t>
         </is>
       </c>
       <c r="B18" s="41" t="n"/>
@@ -13220,87 +13275,89 @@
     <row r="19" ht="20" customHeight="1" s="18">
       <c r="B19" s="42" t="inlineStr">
         <is>
-          <t>Maximum Concurrent Break Ratio</t>
-        </is>
-      </c>
-      <c r="C19" s="46" t="n">
-        <v>0.3</v>
+          <t>Next Sunday Balance Enabled</t>
+        </is>
+      </c>
+      <c r="C19" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="D19" s="44" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1" s="18">
       <c r="B20" s="42" t="inlineStr">
         <is>
-          <t>Maximum Concurrent Breaks</t>
-        </is>
-      </c>
-      <c r="C20" s="45" t="n">
-        <v>4</v>
+          <t>Next Sunday Overage Cap</t>
+        </is>
+      </c>
+      <c r="C20" s="46" t="n">
+        <v>1.3</v>
       </c>
       <c r="D20" s="44" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1" s="18">
       <c r="B21" s="42" t="inlineStr">
         <is>
-          <t>Break Concurrency Gate Mode</t>
-        </is>
-      </c>
-      <c r="C21" s="43" t="inlineStr">
+          <t>Next Sunday Maximum Adjacent Raw Change</t>
+        </is>
+      </c>
+      <c r="C21" s="45" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="44" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" s="18">
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>Next Sunday Balance Gate Mode</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
         <is>
           <t>Warn</t>
         </is>
       </c>
-      <c r="D21" s="44" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="40" t="inlineStr">
-        <is>
-          <t>Week Boundary</t>
-        </is>
-      </c>
-      <c r="B23" s="41" t="n"/>
-      <c r="C23" s="41" t="n"/>
-      <c r="D23" s="41" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" s="18">
-      <c r="B24" s="42" t="inlineStr">
-        <is>
-          <t>Next Sunday Balance Enabled</t>
-        </is>
-      </c>
-      <c r="C24" s="43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D24" s="44" t="inlineStr"/>
+      <c r="D22" s="44" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="40" t="inlineStr">
+        <is>
+          <t>Language / Skill</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="n"/>
+      <c r="C24" s="41" t="n"/>
+      <c r="D24" s="41" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1" s="18">
       <c r="B25" s="42" t="inlineStr">
         <is>
-          <t>Next Sunday Overage Cap</t>
-        </is>
-      </c>
-      <c r="C25" s="46" t="n">
-        <v>1.3</v>
+          <t>Language Operational Reserve Enabled</t>
+        </is>
+      </c>
+      <c r="C25" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="D25" s="44" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1" s="18">
       <c r="B26" s="42" t="inlineStr">
         <is>
-          <t>Next Sunday Maximum Adjacent Raw Change</t>
+          <t>Language Operational Reserve Extra FTE</t>
         </is>
       </c>
       <c r="C26" s="45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D26" s="44" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1" s="18">
       <c r="B27" s="42" t="inlineStr">
         <is>
-          <t>Next Sunday Balance Gate Mode</t>
+          <t>Language Reserve Gate Mode</t>
         </is>
       </c>
       <c r="C27" s="43" t="inlineStr">
@@ -13310,127 +13367,80 @@
       </c>
       <c r="D27" s="44" t="inlineStr"/>
     </row>
-    <row r="29">
-      <c r="A29" s="40" t="inlineStr">
-        <is>
-          <t>Language / Skill</t>
-        </is>
-      </c>
-      <c r="B29" s="41" t="n"/>
-      <c r="C29" s="41" t="n"/>
-      <c r="D29" s="41" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" s="18">
-      <c r="B30" s="42" t="inlineStr">
-        <is>
-          <t>Language Operational Reserve Enabled</t>
-        </is>
-      </c>
-      <c r="C30" s="43" t="inlineStr">
+    <row r="28" ht="20" customHeight="1" s="18">
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>Qualified Language Break Certificate Enabled</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D30" s="44" t="inlineStr"/>
+      <c r="D28" s="44" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="40" t="inlineStr">
+        <is>
+          <t>Whole Week Balance</t>
+        </is>
+      </c>
+      <c r="B30" s="41" t="n"/>
+      <c r="C30" s="41" t="n"/>
+      <c r="D30" s="41" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1" s="18">
       <c r="B31" s="42" t="inlineStr">
         <is>
-          <t>Language Operational Reserve Extra FTE</t>
-        </is>
-      </c>
-      <c r="C31" s="45" t="n">
-        <v>1</v>
+          <t>Whole Week Balance Enabled</t>
+        </is>
+      </c>
+      <c r="C31" s="43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
       <c r="D31" s="44" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1" s="18">
       <c r="B32" s="42" t="inlineStr">
         <is>
-          <t>Language Reserve Gate Mode</t>
-        </is>
-      </c>
-      <c r="C32" s="43" t="inlineStr">
-        <is>
-          <t>Warn</t>
-        </is>
+          <t>Whole Week Overage Cap</t>
+        </is>
+      </c>
+      <c r="C32" s="46" t="n">
+        <v>1.35</v>
       </c>
       <c r="D32" s="44" t="inlineStr"/>
     </row>
-    <row r="33" ht="20" customHeight="1" s="18">
-      <c r="B33" s="42" t="inlineStr">
-        <is>
-          <t>Qualified Language Break Certificate Enabled</t>
-        </is>
-      </c>
-      <c r="C33" s="43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D33" s="44" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="40" t="inlineStr">
-        <is>
-          <t>Whole Week Balance</t>
-        </is>
-      </c>
-      <c r="B35" s="41" t="n"/>
-      <c r="C35" s="41" t="n"/>
-      <c r="D35" s="41" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1" s="18">
-      <c r="B36" s="42" t="inlineStr">
-        <is>
-          <t>Whole Week Balance Enabled</t>
-        </is>
-      </c>
-      <c r="C36" s="43" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D36" s="44" t="inlineStr"/>
-    </row>
-    <row r="37" ht="20" customHeight="1" s="18">
-      <c r="B37" s="42" t="inlineStr">
-        <is>
-          <t>Whole Week Overage Cap</t>
-        </is>
-      </c>
-      <c r="C37" s="46" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="D37" s="44" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="40" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="40" t="inlineStr">
         <is>
           <t>Benchmarks</t>
         </is>
       </c>
-      <c r="B39" s="41" t="n"/>
-      <c r="C39" s="41" t="n"/>
-      <c r="D39" s="41" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1" s="18">
-      <c r="B40" s="42" t="inlineStr">
+      <c r="B34" s="41" t="n"/>
+      <c r="C34" s="41" t="n"/>
+      <c r="D34" s="41" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" s="18">
+      <c r="B35" s="42" t="inlineStr">
         <is>
           <t>Quality Benchmark Tolerance Intervals</t>
         </is>
       </c>
-      <c r="C40" s="45" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="44" t="inlineStr"/>
+      <c r="C35" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="44" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <dataValidations count="17">
+  <dataValidations count="15">
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
@@ -13446,7 +13456,7 @@
       <formula1>0</formula1>
       <formula2>1440</formula2>
     </dataValidation>
-    <dataValidation sqref="C12 C24 C30 C33 C36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+    <dataValidation sqref="C12 C19 C25 C28 C31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="C13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 100% to 500%." prompt="Enter a number from 100% to 500%." type="decimal" errorStyle="stop" operator="between">
@@ -13465,34 +13475,26 @@
       <formula1>0</formula1>
       <formula2>100000000</formula2>
     </dataValidation>
-    <dataValidation sqref="C19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 0% to 100%." prompt="Enter a number from 0% to 100%." type="decimal" errorStyle="stop" operator="between">
-      <formula1>0</formula1>
-      <formula2>1</formula2>
-    </dataValidation>
-    <dataValidation sqref="C20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 1 to 5000." prompt="Enter a whole number from 1 to 5000." type="whole" errorStyle="stop" operator="between">
-      <formula1>1</formula1>
-      <formula2>5000</formula2>
-    </dataValidation>
-    <dataValidation sqref="C21 C27 C32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
-      <formula1>"Warn,Fail,Off"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C25" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 100% to 500%." prompt="Enter a number from 100% to 500%." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="C20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 100% to 500%." prompt="Enter a number from 100% to 500%." type="decimal" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="C26" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 1 to 1000." prompt="Enter a whole number from 1 to 1000." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 1 to 1000." prompt="Enter a whole number from 1 to 1000." type="whole" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>1000</formula2>
     </dataValidation>
-    <dataValidation sqref="C31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 500." prompt="Enter a whole number from 0 to 500." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C22 C27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="Choose a value from the list. Typed values outside the list are not accepted." type="list" errorStyle="stop">
+      <formula1>"Warn,Fail,Off"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C26" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 500." prompt="Enter a whole number from 0 to 500." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>500</formula2>
     </dataValidation>
-    <dataValidation sqref="C37" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 100% to 500%." prompt="Enter a number from 100% to 500%." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="C32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a number from 100% to 500%." prompt="Enter a number from 100% to 500%." type="decimal" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="C40" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
+    <dataValidation sqref="C35" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value not allowed" error="This value is outside what the scheduler accepts. Enter a whole number from 0 to 672." prompt="Enter a whole number from 0 to 672." type="whole" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>672</formula2>
     </dataValidation>

</xml_diff>